<commit_message>
arreglo de tablas de exportacion de coti pdf e implementacion de fotos en el ultimo formato rebo
</commit_message>
<xml_diff>
--- a/public/informes-templates/REPORTE DE BOBINA DE ESTATOR-REBO.xlsx
+++ b/public/informes-templates/REPORTE DE BOBINA DE ESTATOR-REBO.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -716,137 +716,137 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1395,19 +1395,19 @@
   <sheetData>
     <row r="1" spans="3:58" s="67" customFormat="1" ht="11.25" customHeight="1"/>
     <row r="2" spans="3:58" s="67" customFormat="1" ht="11.25" customHeight="1">
-      <c r="AC2" s="114" t="s">
+      <c r="AC2" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="AD2" s="114"/>
-      <c r="AE2" s="114"/>
-      <c r="AF2" s="114"/>
-      <c r="AG2" s="114"/>
-      <c r="AH2" s="114"/>
-      <c r="AI2" s="114"/>
-      <c r="AJ2" s="114"/>
-      <c r="AK2" s="114"/>
-      <c r="AL2" s="114"/>
-      <c r="AM2" s="114"/>
+      <c r="AD2" s="71"/>
+      <c r="AE2" s="71"/>
+      <c r="AF2" s="71"/>
+      <c r="AG2" s="71"/>
+      <c r="AH2" s="71"/>
+      <c r="AI2" s="71"/>
+      <c r="AJ2" s="71"/>
+      <c r="AK2" s="71"/>
+      <c r="AL2" s="71"/>
+      <c r="AM2" s="71"/>
       <c r="AN2" s="70"/>
       <c r="AO2" s="70"/>
       <c r="AR2" s="69"/>
@@ -1427,19 +1427,19 @@
       <c r="BF2" s="69"/>
     </row>
     <row r="3" spans="3:58" s="67" customFormat="1" ht="11.25" customHeight="1">
-      <c r="AC3" s="114" t="s">
+      <c r="AC3" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="AD3" s="114"/>
-      <c r="AE3" s="114"/>
-      <c r="AF3" s="114"/>
-      <c r="AG3" s="114"/>
-      <c r="AH3" s="114"/>
-      <c r="AI3" s="114"/>
-      <c r="AJ3" s="114"/>
-      <c r="AK3" s="114"/>
-      <c r="AL3" s="114"/>
-      <c r="AM3" s="114"/>
+      <c r="AD3" s="71"/>
+      <c r="AE3" s="71"/>
+      <c r="AF3" s="71"/>
+      <c r="AG3" s="71"/>
+      <c r="AH3" s="71"/>
+      <c r="AI3" s="71"/>
+      <c r="AJ3" s="71"/>
+      <c r="AK3" s="71"/>
+      <c r="AL3" s="71"/>
+      <c r="AM3" s="71"/>
       <c r="AN3" s="70"/>
       <c r="AO3" s="70"/>
       <c r="AR3" s="69"/>
@@ -1459,19 +1459,19 @@
       <c r="BF3" s="69"/>
     </row>
     <row r="4" spans="3:58" s="67" customFormat="1" ht="11.25" customHeight="1">
-      <c r="AC4" s="114" t="s">
+      <c r="AC4" s="71" t="s">
         <v>50</v>
       </c>
-      <c r="AD4" s="114"/>
-      <c r="AE4" s="114"/>
-      <c r="AF4" s="114"/>
-      <c r="AG4" s="114"/>
-      <c r="AH4" s="114"/>
-      <c r="AI4" s="114"/>
-      <c r="AJ4" s="114"/>
-      <c r="AK4" s="114"/>
-      <c r="AL4" s="114"/>
-      <c r="AM4" s="114"/>
+      <c r="AD4" s="71"/>
+      <c r="AE4" s="71"/>
+      <c r="AF4" s="71"/>
+      <c r="AG4" s="71"/>
+      <c r="AH4" s="71"/>
+      <c r="AI4" s="71"/>
+      <c r="AJ4" s="71"/>
+      <c r="AK4" s="71"/>
+      <c r="AL4" s="71"/>
+      <c r="AM4" s="71"/>
       <c r="AN4" s="70"/>
       <c r="AO4" s="70"/>
       <c r="AR4" s="69"/>
@@ -1491,19 +1491,19 @@
       <c r="BF4" s="69"/>
     </row>
     <row r="5" spans="3:58" s="67" customFormat="1" ht="11.25" customHeight="1">
-      <c r="AC5" s="114" t="s">
+      <c r="AC5" s="71" t="s">
         <v>51</v>
       </c>
-      <c r="AD5" s="114"/>
-      <c r="AE5" s="114"/>
-      <c r="AF5" s="114"/>
-      <c r="AG5" s="114"/>
-      <c r="AH5" s="114"/>
-      <c r="AI5" s="114"/>
-      <c r="AJ5" s="114"/>
-      <c r="AK5" s="114"/>
-      <c r="AL5" s="114"/>
-      <c r="AM5" s="114"/>
+      <c r="AD5" s="71"/>
+      <c r="AE5" s="71"/>
+      <c r="AF5" s="71"/>
+      <c r="AG5" s="71"/>
+      <c r="AH5" s="71"/>
+      <c r="AI5" s="71"/>
+      <c r="AJ5" s="71"/>
+      <c r="AK5" s="71"/>
+      <c r="AL5" s="71"/>
+      <c r="AM5" s="71"/>
       <c r="AN5" s="70"/>
       <c r="AO5" s="70"/>
       <c r="AR5" s="69"/>
@@ -1523,19 +1523,19 @@
       <c r="BF5" s="69"/>
     </row>
     <row r="6" spans="3:58" s="67" customFormat="1" ht="11.25" customHeight="1">
-      <c r="AC6" s="114" t="s">
+      <c r="AC6" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="AD6" s="114"/>
-      <c r="AE6" s="114"/>
-      <c r="AF6" s="114"/>
-      <c r="AG6" s="114"/>
-      <c r="AH6" s="114"/>
-      <c r="AI6" s="114"/>
-      <c r="AJ6" s="114"/>
-      <c r="AK6" s="114"/>
-      <c r="AL6" s="114"/>
-      <c r="AM6" s="114"/>
+      <c r="AD6" s="71"/>
+      <c r="AE6" s="71"/>
+      <c r="AF6" s="71"/>
+      <c r="AG6" s="71"/>
+      <c r="AH6" s="71"/>
+      <c r="AI6" s="71"/>
+      <c r="AJ6" s="71"/>
+      <c r="AK6" s="71"/>
+      <c r="AL6" s="71"/>
+      <c r="AM6" s="71"/>
       <c r="AN6" s="70"/>
       <c r="AO6" s="70"/>
       <c r="AR6" s="69"/>
@@ -1586,40 +1586,40 @@
     <row r="9" spans="3:58" ht="11.25" customHeight="1">
       <c r="C9" s="2"/>
       <c r="D9" s="37"/>
-      <c r="E9" s="110" t="s">
+      <c r="E9" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="111"/>
-      <c r="G9" s="111"/>
-      <c r="H9" s="111"/>
-      <c r="I9" s="111"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="111"/>
-      <c r="L9" s="111"/>
-      <c r="M9" s="111"/>
-      <c r="N9" s="111"/>
-      <c r="O9" s="111"/>
-      <c r="P9" s="111"/>
-      <c r="Q9" s="111"/>
-      <c r="R9" s="111"/>
-      <c r="S9" s="111"/>
-      <c r="T9" s="111"/>
-      <c r="U9" s="111"/>
-      <c r="V9" s="111"/>
-      <c r="W9" s="111"/>
-      <c r="X9" s="111"/>
-      <c r="Y9" s="111"/>
-      <c r="Z9" s="111"/>
-      <c r="AA9" s="111"/>
-      <c r="AB9" s="111"/>
-      <c r="AC9" s="111"/>
-      <c r="AD9" s="111"/>
-      <c r="AE9" s="111"/>
-      <c r="AF9" s="111"/>
-      <c r="AG9" s="111"/>
-      <c r="AH9" s="111"/>
-      <c r="AI9" s="111"/>
-      <c r="AJ9" s="112"/>
+      <c r="F9" s="82"/>
+      <c r="G9" s="82"/>
+      <c r="H9" s="82"/>
+      <c r="I9" s="82"/>
+      <c r="J9" s="82"/>
+      <c r="K9" s="82"/>
+      <c r="L9" s="82"/>
+      <c r="M9" s="82"/>
+      <c r="N9" s="82"/>
+      <c r="O9" s="82"/>
+      <c r="P9" s="82"/>
+      <c r="Q9" s="82"/>
+      <c r="R9" s="82"/>
+      <c r="S9" s="82"/>
+      <c r="T9" s="82"/>
+      <c r="U9" s="82"/>
+      <c r="V9" s="82"/>
+      <c r="W9" s="82"/>
+      <c r="X9" s="82"/>
+      <c r="Y9" s="82"/>
+      <c r="Z9" s="82"/>
+      <c r="AA9" s="82"/>
+      <c r="AB9" s="82"/>
+      <c r="AC9" s="82"/>
+      <c r="AD9" s="82"/>
+      <c r="AE9" s="82"/>
+      <c r="AF9" s="82"/>
+      <c r="AG9" s="82"/>
+      <c r="AH9" s="82"/>
+      <c r="AI9" s="82"/>
+      <c r="AJ9" s="83"/>
       <c r="AK9" s="37"/>
       <c r="AL9" s="37"/>
     </row>
@@ -1662,29 +1662,29 @@
       <c r="AL10" s="38"/>
     </row>
     <row r="11" spans="3:58" ht="11.25" customHeight="1">
-      <c r="C11" s="103" t="s">
+      <c r="C11" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="103"/>
-      <c r="E11" s="103"/>
-      <c r="F11" s="103"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="74"/>
-      <c r="J11" s="74"/>
-      <c r="K11" s="74"/>
-      <c r="L11" s="74"/>
-      <c r="M11" s="74"/>
-      <c r="N11" s="74"/>
-      <c r="O11" s="74"/>
-      <c r="P11" s="74"/>
-      <c r="Q11" s="75"/>
-      <c r="R11" s="103" t="s">
+      <c r="D11" s="80"/>
+      <c r="E11" s="80"/>
+      <c r="F11" s="80"/>
+      <c r="G11" s="85"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="86"/>
+      <c r="J11" s="86"/>
+      <c r="K11" s="86"/>
+      <c r="L11" s="86"/>
+      <c r="M11" s="86"/>
+      <c r="N11" s="86"/>
+      <c r="O11" s="86"/>
+      <c r="P11" s="86"/>
+      <c r="Q11" s="87"/>
+      <c r="R11" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="S11" s="103"/>
-      <c r="T11" s="103"/>
-      <c r="U11" s="103"/>
+      <c r="S11" s="80"/>
+      <c r="T11" s="80"/>
+      <c r="U11" s="80"/>
       <c r="V11" s="79"/>
       <c r="W11" s="79"/>
       <c r="X11" s="79"/>
@@ -1695,40 +1695,40 @@
       <c r="AC11" s="79"/>
       <c r="AD11" s="79"/>
       <c r="AE11" s="79"/>
-      <c r="AF11" s="103" t="s">
+      <c r="AF11" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="AG11" s="103"/>
-      <c r="AH11" s="103"/>
-      <c r="AI11" s="108"/>
-      <c r="AJ11" s="108"/>
-      <c r="AK11" s="108"/>
-      <c r="AL11" s="108"/>
+      <c r="AG11" s="80"/>
+      <c r="AH11" s="80"/>
+      <c r="AI11" s="88"/>
+      <c r="AJ11" s="88"/>
+      <c r="AK11" s="88"/>
+      <c r="AL11" s="88"/>
     </row>
     <row r="12" spans="3:58" ht="11.25" customHeight="1">
-      <c r="C12" s="103" t="s">
+      <c r="C12" s="80" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="103"/>
-      <c r="E12" s="103"/>
-      <c r="F12" s="103"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="74"/>
-      <c r="I12" s="74"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="74"/>
-      <c r="L12" s="74"/>
-      <c r="M12" s="74"/>
-      <c r="N12" s="74"/>
-      <c r="O12" s="74"/>
-      <c r="P12" s="74"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="103" t="s">
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
+      <c r="F12" s="80"/>
+      <c r="G12" s="85"/>
+      <c r="H12" s="86"/>
+      <c r="I12" s="86"/>
+      <c r="J12" s="86"/>
+      <c r="K12" s="86"/>
+      <c r="L12" s="86"/>
+      <c r="M12" s="86"/>
+      <c r="N12" s="86"/>
+      <c r="O12" s="86"/>
+      <c r="P12" s="86"/>
+      <c r="Q12" s="87"/>
+      <c r="R12" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="S12" s="103"/>
-      <c r="T12" s="103"/>
-      <c r="U12" s="103"/>
+      <c r="S12" s="80"/>
+      <c r="T12" s="80"/>
+      <c r="U12" s="80"/>
       <c r="V12" s="79"/>
       <c r="W12" s="79"/>
       <c r="X12" s="79"/>
@@ -1739,15 +1739,15 @@
       <c r="AC12" s="79"/>
       <c r="AD12" s="79"/>
       <c r="AE12" s="79"/>
-      <c r="AF12" s="104" t="s">
+      <c r="AF12" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="AG12" s="104"/>
-      <c r="AH12" s="104"/>
-      <c r="AI12" s="87"/>
-      <c r="AJ12" s="87"/>
-      <c r="AK12" s="87"/>
-      <c r="AL12" s="87"/>
+      <c r="AG12" s="84"/>
+      <c r="AH12" s="84"/>
+      <c r="AI12" s="77"/>
+      <c r="AJ12" s="77"/>
+      <c r="AK12" s="77"/>
+      <c r="AL12" s="77"/>
     </row>
     <row r="13" spans="3:58" ht="11.25" customHeight="1">
       <c r="C13" s="2"/>
@@ -1788,46 +1788,46 @@
       <c r="AL13" s="33"/>
     </row>
     <row r="14" spans="3:58" ht="11.25" customHeight="1">
-      <c r="C14" s="76" t="s">
+      <c r="C14" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="77"/>
-      <c r="E14" s="77"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="77"/>
-      <c r="H14" s="77"/>
-      <c r="I14" s="77"/>
-      <c r="J14" s="77"/>
-      <c r="K14" s="77"/>
-      <c r="L14" s="77"/>
-      <c r="M14" s="77"/>
-      <c r="N14" s="77"/>
-      <c r="O14" s="77"/>
-      <c r="P14" s="77"/>
-      <c r="Q14" s="77"/>
-      <c r="R14" s="77"/>
-      <c r="S14" s="77"/>
-      <c r="T14" s="78"/>
-      <c r="U14" s="76" t="s">
+      <c r="D14" s="73"/>
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="73"/>
+      <c r="I14" s="73"/>
+      <c r="J14" s="73"/>
+      <c r="K14" s="73"/>
+      <c r="L14" s="73"/>
+      <c r="M14" s="73"/>
+      <c r="N14" s="73"/>
+      <c r="O14" s="73"/>
+      <c r="P14" s="73"/>
+      <c r="Q14" s="73"/>
+      <c r="R14" s="73"/>
+      <c r="S14" s="73"/>
+      <c r="T14" s="74"/>
+      <c r="U14" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="V14" s="77"/>
-      <c r="W14" s="77"/>
-      <c r="X14" s="77"/>
-      <c r="Y14" s="77"/>
-      <c r="Z14" s="77"/>
-      <c r="AA14" s="77"/>
-      <c r="AB14" s="77"/>
-      <c r="AC14" s="77"/>
-      <c r="AD14" s="77"/>
-      <c r="AE14" s="77"/>
-      <c r="AF14" s="77"/>
-      <c r="AG14" s="77"/>
-      <c r="AH14" s="77"/>
-      <c r="AI14" s="77"/>
-      <c r="AJ14" s="77"/>
-      <c r="AK14" s="77"/>
-      <c r="AL14" s="78"/>
+      <c r="V14" s="73"/>
+      <c r="W14" s="73"/>
+      <c r="X14" s="73"/>
+      <c r="Y14" s="73"/>
+      <c r="Z14" s="73"/>
+      <c r="AA14" s="73"/>
+      <c r="AB14" s="73"/>
+      <c r="AC14" s="73"/>
+      <c r="AD14" s="73"/>
+      <c r="AE14" s="73"/>
+      <c r="AF14" s="73"/>
+      <c r="AG14" s="73"/>
+      <c r="AH14" s="73"/>
+      <c r="AI14" s="73"/>
+      <c r="AJ14" s="73"/>
+      <c r="AK14" s="73"/>
+      <c r="AL14" s="74"/>
     </row>
     <row r="15" spans="3:58" ht="11.25" customHeight="1">
       <c r="C15" s="60"/>
@@ -1916,11 +1916,11 @@
       <c r="L17" s="21"/>
       <c r="M17" s="21"/>
       <c r="N17" s="21"/>
-      <c r="O17" s="113"/>
-      <c r="P17" s="113"/>
-      <c r="Q17" s="113"/>
-      <c r="R17" s="113"/>
-      <c r="S17" s="113"/>
+      <c r="O17" s="75"/>
+      <c r="P17" s="75"/>
+      <c r="Q17" s="75"/>
+      <c r="R17" s="75"/>
+      <c r="S17" s="75"/>
       <c r="T17" s="21"/>
       <c r="U17" s="20"/>
       <c r="V17" s="21"/>
@@ -1949,9 +1949,9 @@
       <c r="E18" s="21"/>
       <c r="F18" s="21"/>
       <c r="G18" s="21"/>
-      <c r="H18" s="109"/>
-      <c r="I18" s="109"/>
-      <c r="J18" s="109"/>
+      <c r="H18" s="76"/>
+      <c r="I18" s="76"/>
+      <c r="J18" s="76"/>
       <c r="K18" s="21"/>
       <c r="L18" s="21"/>
       <c r="M18" s="21"/>
@@ -1985,9 +1985,9 @@
       <c r="E19" s="21"/>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="109"/>
-      <c r="I19" s="109"/>
-      <c r="J19" s="109"/>
+      <c r="H19" s="76"/>
+      <c r="I19" s="76"/>
+      <c r="J19" s="76"/>
       <c r="K19" s="21"/>
       <c r="L19" s="21"/>
       <c r="M19" s="21"/>
@@ -2345,19 +2345,19 @@
       <c r="C29" s="40"/>
       <c r="D29" s="21"/>
       <c r="E29" s="2"/>
-      <c r="F29" s="80" t="s">
+      <c r="F29" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="G29" s="80"/>
-      <c r="H29" s="80"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
       <c r="I29" s="79"/>
       <c r="J29" s="79"/>
       <c r="K29" s="79"/>
-      <c r="L29" s="80" t="s">
+      <c r="L29" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="M29" s="80"/>
-      <c r="N29" s="80"/>
+      <c r="M29" s="78"/>
+      <c r="N29" s="78"/>
       <c r="O29" s="79"/>
       <c r="P29" s="79"/>
       <c r="Q29" s="79"/>
@@ -2387,19 +2387,19 @@
       <c r="C30" s="40"/>
       <c r="D30" s="21"/>
       <c r="E30" s="2"/>
-      <c r="F30" s="80" t="s">
+      <c r="F30" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="G30" s="80"/>
-      <c r="H30" s="80"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="78"/>
       <c r="I30" s="79"/>
       <c r="J30" s="79"/>
       <c r="K30" s="79"/>
-      <c r="L30" s="80" t="s">
+      <c r="L30" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="M30" s="80"/>
-      <c r="N30" s="80"/>
+      <c r="M30" s="78"/>
+      <c r="N30" s="78"/>
       <c r="O30" s="79"/>
       <c r="P30" s="79"/>
       <c r="Q30" s="79"/>
@@ -2507,22 +2507,22 @@
       <c r="C33" s="40"/>
       <c r="D33" s="21"/>
       <c r="E33" s="2"/>
-      <c r="F33" s="76" t="s">
+      <c r="F33" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="G33" s="77"/>
-      <c r="H33" s="78"/>
-      <c r="I33" s="73"/>
-      <c r="J33" s="74"/>
-      <c r="K33" s="75"/>
-      <c r="L33" s="76" t="s">
+      <c r="G33" s="73"/>
+      <c r="H33" s="74"/>
+      <c r="I33" s="85"/>
+      <c r="J33" s="86"/>
+      <c r="K33" s="87"/>
+      <c r="L33" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="M33" s="77"/>
-      <c r="N33" s="78"/>
-      <c r="O33" s="73"/>
-      <c r="P33" s="74"/>
-      <c r="Q33" s="75"/>
+      <c r="M33" s="73"/>
+      <c r="N33" s="74"/>
+      <c r="O33" s="85"/>
+      <c r="P33" s="86"/>
+      <c r="Q33" s="87"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
       <c r="T33" s="48"/>
@@ -2549,22 +2549,22 @@
       <c r="C34" s="40"/>
       <c r="D34" s="21"/>
       <c r="E34" s="2"/>
-      <c r="F34" s="76" t="s">
+      <c r="F34" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="G34" s="77"/>
-      <c r="H34" s="78"/>
-      <c r="I34" s="73"/>
-      <c r="J34" s="74"/>
-      <c r="K34" s="75"/>
-      <c r="L34" s="76" t="s">
+      <c r="G34" s="73"/>
+      <c r="H34" s="74"/>
+      <c r="I34" s="85"/>
+      <c r="J34" s="86"/>
+      <c r="K34" s="87"/>
+      <c r="L34" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="M34" s="77"/>
-      <c r="N34" s="78"/>
-      <c r="O34" s="73"/>
-      <c r="P34" s="74"/>
-      <c r="Q34" s="75"/>
+      <c r="M34" s="73"/>
+      <c r="N34" s="74"/>
+      <c r="O34" s="85"/>
+      <c r="P34" s="86"/>
+      <c r="Q34" s="87"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
       <c r="T34" s="48"/>
@@ -2592,22 +2592,22 @@
       <c r="C35" s="40"/>
       <c r="D35" s="21"/>
       <c r="E35" s="2"/>
-      <c r="F35" s="76" t="s">
+      <c r="F35" s="72" t="s">
         <v>20</v>
       </c>
-      <c r="G35" s="77"/>
-      <c r="H35" s="78"/>
-      <c r="I35" s="73"/>
-      <c r="J35" s="74"/>
-      <c r="K35" s="75"/>
-      <c r="L35" s="76" t="s">
+      <c r="G35" s="73"/>
+      <c r="H35" s="74"/>
+      <c r="I35" s="85"/>
+      <c r="J35" s="86"/>
+      <c r="K35" s="87"/>
+      <c r="L35" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="M35" s="77"/>
-      <c r="N35" s="78"/>
-      <c r="O35" s="73"/>
-      <c r="P35" s="74"/>
-      <c r="Q35" s="75"/>
+      <c r="M35" s="73"/>
+      <c r="N35" s="74"/>
+      <c r="O35" s="85"/>
+      <c r="P35" s="86"/>
+      <c r="Q35" s="87"/>
       <c r="R35" s="2"/>
       <c r="S35" s="2"/>
       <c r="T35" s="48"/>
@@ -2719,19 +2719,19 @@
       <c r="C38" s="40"/>
       <c r="D38" s="21"/>
       <c r="E38" s="2"/>
-      <c r="F38" s="76" t="s">
+      <c r="F38" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="G38" s="77"/>
-      <c r="H38" s="78"/>
-      <c r="I38" s="73"/>
-      <c r="J38" s="74"/>
-      <c r="K38" s="75"/>
-      <c r="L38" s="76" t="s">
+      <c r="G38" s="73"/>
+      <c r="H38" s="74"/>
+      <c r="I38" s="85"/>
+      <c r="J38" s="86"/>
+      <c r="K38" s="87"/>
+      <c r="L38" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="M38" s="77"/>
-      <c r="N38" s="78"/>
+      <c r="M38" s="73"/>
+      <c r="N38" s="74"/>
       <c r="O38" s="79"/>
       <c r="P38" s="79"/>
       <c r="Q38" s="79"/>
@@ -2764,19 +2764,19 @@
       <c r="C39" s="43"/>
       <c r="D39" s="21"/>
       <c r="E39" s="2"/>
-      <c r="F39" s="76" t="s">
+      <c r="F39" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="G39" s="77"/>
-      <c r="H39" s="78"/>
-      <c r="I39" s="73"/>
-      <c r="J39" s="74"/>
-      <c r="K39" s="75"/>
-      <c r="L39" s="76" t="s">
+      <c r="G39" s="73"/>
+      <c r="H39" s="74"/>
+      <c r="I39" s="85"/>
+      <c r="J39" s="86"/>
+      <c r="K39" s="87"/>
+      <c r="L39" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="M39" s="77"/>
-      <c r="N39" s="78"/>
+      <c r="M39" s="73"/>
+      <c r="N39" s="74"/>
       <c r="O39" s="79"/>
       <c r="P39" s="79"/>
       <c r="Q39" s="79"/>
@@ -2809,19 +2809,19 @@
       <c r="C40" s="40"/>
       <c r="D40" s="21"/>
       <c r="E40" s="2"/>
-      <c r="F40" s="80" t="s">
+      <c r="F40" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="G40" s="80"/>
-      <c r="H40" s="80"/>
+      <c r="G40" s="78"/>
+      <c r="H40" s="78"/>
       <c r="I40" s="79"/>
       <c r="J40" s="79"/>
       <c r="K40" s="79"/>
-      <c r="L40" s="76" t="s">
+      <c r="L40" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="M40" s="77"/>
-      <c r="N40" s="78"/>
+      <c r="M40" s="73"/>
+      <c r="N40" s="74"/>
       <c r="O40" s="79"/>
       <c r="P40" s="79"/>
       <c r="Q40" s="79"/>
@@ -2927,20 +2927,20 @@
         <v>39</v>
       </c>
       <c r="E43" s="2"/>
-      <c r="F43" s="71"/>
-      <c r="G43" s="71"/>
-      <c r="H43" s="71"/>
-      <c r="I43" s="71"/>
-      <c r="J43" s="71"/>
-      <c r="K43" s="71"/>
+      <c r="F43" s="113"/>
+      <c r="G43" s="113"/>
+      <c r="H43" s="113"/>
+      <c r="I43" s="113"/>
+      <c r="J43" s="113"/>
+      <c r="K43" s="113"/>
       <c r="L43" s="66" t="s">
         <v>45</v>
       </c>
       <c r="O43" s="2"/>
-      <c r="P43" s="71"/>
-      <c r="Q43" s="71"/>
-      <c r="R43" s="71"/>
-      <c r="S43" s="71"/>
+      <c r="P43" s="113"/>
+      <c r="Q43" s="113"/>
+      <c r="R43" s="113"/>
+      <c r="S43" s="113"/>
       <c r="T43" s="48"/>
       <c r="U43" s="35" t="s">
         <v>7</v>
@@ -2975,20 +2975,20 @@
       </c>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
-      <c r="G44" s="71"/>
-      <c r="H44" s="71"/>
-      <c r="I44" s="71"/>
-      <c r="J44" s="71"/>
-      <c r="K44" s="71"/>
+      <c r="G44" s="113"/>
+      <c r="H44" s="113"/>
+      <c r="I44" s="113"/>
+      <c r="J44" s="113"/>
+      <c r="K44" s="113"/>
       <c r="L44" s="65" t="s">
         <v>47</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
-      <c r="Q44" s="71"/>
-      <c r="R44" s="71"/>
-      <c r="S44" s="71"/>
+      <c r="Q44" s="113"/>
+      <c r="R44" s="113"/>
+      <c r="S44" s="113"/>
       <c r="T44" s="48"/>
       <c r="U44" s="35" t="s">
         <v>7</v>
@@ -3023,20 +3023,20 @@
       </c>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="71"/>
-      <c r="H45" s="71"/>
-      <c r="I45" s="71"/>
-      <c r="J45" s="71"/>
-      <c r="K45" s="71"/>
+      <c r="G45" s="113"/>
+      <c r="H45" s="113"/>
+      <c r="I45" s="113"/>
+      <c r="J45" s="113"/>
+      <c r="K45" s="113"/>
       <c r="L45" s="65" t="s">
         <v>46</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
-      <c r="Q45" s="71"/>
-      <c r="R45" s="71"/>
-      <c r="S45" s="71"/>
+      <c r="Q45" s="113"/>
+      <c r="R45" s="113"/>
+      <c r="S45" s="113"/>
       <c r="T45" s="48"/>
       <c r="U45" s="35" t="s">
         <v>7</v>
@@ -3070,18 +3070,18 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
-      <c r="H46" s="71"/>
-      <c r="I46" s="71"/>
-      <c r="J46" s="71"/>
-      <c r="K46" s="71"/>
-      <c r="L46" s="71"/>
-      <c r="M46" s="71"/>
-      <c r="N46" s="71"/>
-      <c r="O46" s="71"/>
-      <c r="P46" s="71"/>
-      <c r="Q46" s="71"/>
-      <c r="R46" s="71"/>
-      <c r="S46" s="71"/>
+      <c r="H46" s="113"/>
+      <c r="I46" s="113"/>
+      <c r="J46" s="113"/>
+      <c r="K46" s="113"/>
+      <c r="L46" s="113"/>
+      <c r="M46" s="113"/>
+      <c r="N46" s="113"/>
+      <c r="O46" s="113"/>
+      <c r="P46" s="113"/>
+      <c r="Q46" s="113"/>
+      <c r="R46" s="113"/>
+      <c r="S46" s="113"/>
       <c r="T46" s="48"/>
       <c r="U46" s="35" t="s">
         <v>7</v>
@@ -3106,15 +3106,15 @@
       <c r="D47" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="K47" s="72"/>
-      <c r="L47" s="72"/>
-      <c r="M47" s="72"/>
-      <c r="N47" s="72"/>
-      <c r="O47" s="72"/>
-      <c r="P47" s="72"/>
-      <c r="Q47" s="72"/>
-      <c r="R47" s="72"/>
-      <c r="S47" s="72"/>
+      <c r="K47" s="114"/>
+      <c r="L47" s="114"/>
+      <c r="M47" s="114"/>
+      <c r="N47" s="114"/>
+      <c r="O47" s="114"/>
+      <c r="P47" s="114"/>
+      <c r="Q47" s="114"/>
+      <c r="R47" s="114"/>
+      <c r="S47" s="114"/>
       <c r="T47" s="8"/>
       <c r="U47" s="35" t="s">
         <v>7</v>
@@ -3142,15 +3142,15 @@
       <c r="D48" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="K48" s="72"/>
-      <c r="L48" s="72"/>
-      <c r="M48" s="72"/>
-      <c r="N48" s="72"/>
-      <c r="O48" s="72"/>
-      <c r="P48" s="72"/>
-      <c r="Q48" s="72"/>
-      <c r="R48" s="72"/>
-      <c r="S48" s="72"/>
+      <c r="K48" s="114"/>
+      <c r="L48" s="114"/>
+      <c r="M48" s="114"/>
+      <c r="N48" s="114"/>
+      <c r="O48" s="114"/>
+      <c r="P48" s="114"/>
+      <c r="Q48" s="114"/>
+      <c r="R48" s="114"/>
+      <c r="S48" s="114"/>
       <c r="T48" s="8"/>
       <c r="AL48" s="8"/>
     </row>
@@ -4302,40 +4302,40 @@
     <row r="80" spans="3:38" ht="11.25" customHeight="1"/>
     <row r="81" spans="3:38" ht="11.25" customHeight="1">
       <c r="D81" s="11"/>
-      <c r="E81" s="105" t="s">
+      <c r="E81" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="F81" s="106"/>
-      <c r="G81" s="106"/>
-      <c r="H81" s="106"/>
-      <c r="I81" s="106"/>
-      <c r="J81" s="106"/>
-      <c r="K81" s="106"/>
-      <c r="L81" s="106"/>
-      <c r="M81" s="106"/>
-      <c r="N81" s="106"/>
-      <c r="O81" s="106"/>
-      <c r="P81" s="106"/>
-      <c r="Q81" s="106"/>
-      <c r="R81" s="106"/>
-      <c r="S81" s="106"/>
-      <c r="T81" s="106"/>
-      <c r="U81" s="106"/>
-      <c r="V81" s="106"/>
-      <c r="W81" s="106"/>
-      <c r="X81" s="106"/>
-      <c r="Y81" s="106"/>
-      <c r="Z81" s="106"/>
-      <c r="AA81" s="106"/>
-      <c r="AB81" s="106"/>
-      <c r="AC81" s="106"/>
-      <c r="AD81" s="106"/>
-      <c r="AE81" s="106"/>
-      <c r="AF81" s="106"/>
-      <c r="AG81" s="106"/>
-      <c r="AH81" s="106"/>
-      <c r="AI81" s="106"/>
-      <c r="AJ81" s="107"/>
+      <c r="F81" s="90"/>
+      <c r="G81" s="90"/>
+      <c r="H81" s="90"/>
+      <c r="I81" s="90"/>
+      <c r="J81" s="90"/>
+      <c r="K81" s="90"/>
+      <c r="L81" s="90"/>
+      <c r="M81" s="90"/>
+      <c r="N81" s="90"/>
+      <c r="O81" s="90"/>
+      <c r="P81" s="90"/>
+      <c r="Q81" s="90"/>
+      <c r="R81" s="90"/>
+      <c r="S81" s="90"/>
+      <c r="T81" s="90"/>
+      <c r="U81" s="90"/>
+      <c r="V81" s="90"/>
+      <c r="W81" s="90"/>
+      <c r="X81" s="90"/>
+      <c r="Y81" s="90"/>
+      <c r="Z81" s="90"/>
+      <c r="AA81" s="90"/>
+      <c r="AB81" s="90"/>
+      <c r="AC81" s="90"/>
+      <c r="AD81" s="90"/>
+      <c r="AE81" s="90"/>
+      <c r="AF81" s="90"/>
+      <c r="AG81" s="90"/>
+      <c r="AH81" s="90"/>
+      <c r="AI81" s="90"/>
+      <c r="AJ81" s="91"/>
       <c r="AK81" s="11"/>
       <c r="AL81" s="11"/>
     </row>
@@ -4377,32 +4377,32 @@
       <c r="AL82" s="12"/>
     </row>
     <row r="83" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C83" s="103" t="s">
+      <c r="C83" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="D83" s="103"/>
-      <c r="E83" s="103"/>
-      <c r="F83" s="103"/>
-      <c r="G83" s="73">
+      <c r="D83" s="80"/>
+      <c r="E83" s="80"/>
+      <c r="F83" s="80"/>
+      <c r="G83" s="85">
         <f>G11</f>
         <v>0</v>
       </c>
-      <c r="H83" s="74"/>
-      <c r="I83" s="74"/>
-      <c r="J83" s="74"/>
-      <c r="K83" s="74"/>
-      <c r="L83" s="74"/>
-      <c r="M83" s="74"/>
-      <c r="N83" s="74"/>
-      <c r="O83" s="74"/>
-      <c r="P83" s="74"/>
-      <c r="Q83" s="75"/>
-      <c r="R83" s="103" t="s">
+      <c r="H83" s="86"/>
+      <c r="I83" s="86"/>
+      <c r="J83" s="86"/>
+      <c r="K83" s="86"/>
+      <c r="L83" s="86"/>
+      <c r="M83" s="86"/>
+      <c r="N83" s="86"/>
+      <c r="O83" s="86"/>
+      <c r="P83" s="86"/>
+      <c r="Q83" s="87"/>
+      <c r="R83" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="S83" s="103"/>
-      <c r="T83" s="103"/>
-      <c r="U83" s="103"/>
+      <c r="S83" s="80"/>
+      <c r="T83" s="80"/>
+      <c r="U83" s="80"/>
       <c r="V83" s="79">
         <f>V11</f>
         <v>0</v>
@@ -4416,46 +4416,46 @@
       <c r="AC83" s="79"/>
       <c r="AD83" s="79"/>
       <c r="AE83" s="79"/>
-      <c r="AF83" s="103" t="s">
+      <c r="AF83" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="AG83" s="103"/>
-      <c r="AH83" s="103"/>
-      <c r="AI83" s="108">
+      <c r="AG83" s="80"/>
+      <c r="AH83" s="80"/>
+      <c r="AI83" s="88">
         <f>AI11</f>
         <v>0</v>
       </c>
-      <c r="AJ83" s="108"/>
-      <c r="AK83" s="108"/>
-      <c r="AL83" s="108"/>
+      <c r="AJ83" s="88"/>
+      <c r="AK83" s="88"/>
+      <c r="AL83" s="88"/>
     </row>
     <row r="84" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C84" s="103" t="s">
+      <c r="C84" s="80" t="s">
         <v>8</v>
       </c>
-      <c r="D84" s="103"/>
-      <c r="E84" s="103"/>
-      <c r="F84" s="103"/>
-      <c r="G84" s="73">
+      <c r="D84" s="80"/>
+      <c r="E84" s="80"/>
+      <c r="F84" s="80"/>
+      <c r="G84" s="85">
         <f>G12</f>
         <v>0</v>
       </c>
-      <c r="H84" s="74"/>
-      <c r="I84" s="74"/>
-      <c r="J84" s="74"/>
-      <c r="K84" s="74"/>
-      <c r="L84" s="74"/>
-      <c r="M84" s="74"/>
-      <c r="N84" s="74"/>
-      <c r="O84" s="74"/>
-      <c r="P84" s="74"/>
-      <c r="Q84" s="75"/>
-      <c r="R84" s="103" t="s">
+      <c r="H84" s="86"/>
+      <c r="I84" s="86"/>
+      <c r="J84" s="86"/>
+      <c r="K84" s="86"/>
+      <c r="L84" s="86"/>
+      <c r="M84" s="86"/>
+      <c r="N84" s="86"/>
+      <c r="O84" s="86"/>
+      <c r="P84" s="86"/>
+      <c r="Q84" s="87"/>
+      <c r="R84" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="S84" s="103"/>
-      <c r="T84" s="103"/>
-      <c r="U84" s="103"/>
+      <c r="S84" s="80"/>
+      <c r="T84" s="80"/>
+      <c r="U84" s="80"/>
       <c r="V84" s="79">
         <f>V12</f>
         <v>0</v>
@@ -4469,18 +4469,18 @@
       <c r="AC84" s="79"/>
       <c r="AD84" s="79"/>
       <c r="AE84" s="79"/>
-      <c r="AF84" s="104" t="s">
+      <c r="AF84" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="AG84" s="104"/>
-      <c r="AH84" s="104"/>
-      <c r="AI84" s="87">
+      <c r="AG84" s="84"/>
+      <c r="AH84" s="84"/>
+      <c r="AI84" s="77">
         <f>AI12</f>
         <v>0</v>
       </c>
-      <c r="AJ84" s="87"/>
-      <c r="AK84" s="87"/>
-      <c r="AL84" s="87"/>
+      <c r="AJ84" s="77"/>
+      <c r="AK84" s="77"/>
+      <c r="AL84" s="77"/>
     </row>
     <row r="85" spans="3:38" ht="11.25" customHeight="1">
       <c r="D85" s="1"/>
@@ -4520,82 +4520,82 @@
       <c r="AL85" s="1"/>
     </row>
     <row r="86" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C86" s="88" t="s">
+      <c r="C86" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="D86" s="89"/>
-      <c r="E86" s="89"/>
-      <c r="F86" s="89"/>
-      <c r="G86" s="89"/>
-      <c r="H86" s="89"/>
-      <c r="I86" s="89"/>
-      <c r="J86" s="89"/>
-      <c r="K86" s="89"/>
-      <c r="L86" s="89"/>
-      <c r="M86" s="89"/>
-      <c r="N86" s="89"/>
-      <c r="O86" s="89"/>
-      <c r="P86" s="89"/>
-      <c r="Q86" s="89"/>
-      <c r="R86" s="89"/>
-      <c r="S86" s="89"/>
-      <c r="T86" s="89"/>
-      <c r="U86" s="89"/>
-      <c r="V86" s="89"/>
-      <c r="W86" s="89"/>
-      <c r="X86" s="89"/>
-      <c r="Y86" s="89"/>
-      <c r="Z86" s="89"/>
-      <c r="AA86" s="89"/>
-      <c r="AB86" s="89"/>
-      <c r="AC86" s="89"/>
-      <c r="AD86" s="89"/>
-      <c r="AE86" s="89"/>
-      <c r="AF86" s="89"/>
-      <c r="AG86" s="89"/>
-      <c r="AH86" s="89"/>
-      <c r="AI86" s="89"/>
-      <c r="AJ86" s="89"/>
-      <c r="AK86" s="89"/>
-      <c r="AL86" s="90"/>
+      <c r="D86" s="99"/>
+      <c r="E86" s="99"/>
+      <c r="F86" s="99"/>
+      <c r="G86" s="99"/>
+      <c r="H86" s="99"/>
+      <c r="I86" s="99"/>
+      <c r="J86" s="99"/>
+      <c r="K86" s="99"/>
+      <c r="L86" s="99"/>
+      <c r="M86" s="99"/>
+      <c r="N86" s="99"/>
+      <c r="O86" s="99"/>
+      <c r="P86" s="99"/>
+      <c r="Q86" s="99"/>
+      <c r="R86" s="99"/>
+      <c r="S86" s="99"/>
+      <c r="T86" s="99"/>
+      <c r="U86" s="99"/>
+      <c r="V86" s="99"/>
+      <c r="W86" s="99"/>
+      <c r="X86" s="99"/>
+      <c r="Y86" s="99"/>
+      <c r="Z86" s="99"/>
+      <c r="AA86" s="99"/>
+      <c r="AB86" s="99"/>
+      <c r="AC86" s="99"/>
+      <c r="AD86" s="99"/>
+      <c r="AE86" s="99"/>
+      <c r="AF86" s="99"/>
+      <c r="AG86" s="99"/>
+      <c r="AH86" s="99"/>
+      <c r="AI86" s="99"/>
+      <c r="AJ86" s="99"/>
+      <c r="AK86" s="99"/>
+      <c r="AL86" s="100"/>
     </row>
     <row r="87" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C87" s="91"/>
-      <c r="D87" s="92"/>
-      <c r="E87" s="92"/>
-      <c r="F87" s="92"/>
-      <c r="G87" s="92"/>
-      <c r="H87" s="92"/>
-      <c r="I87" s="92"/>
-      <c r="J87" s="92"/>
-      <c r="K87" s="92"/>
-      <c r="L87" s="92"/>
-      <c r="M87" s="92"/>
-      <c r="N87" s="92"/>
-      <c r="O87" s="92"/>
-      <c r="P87" s="92"/>
-      <c r="Q87" s="92"/>
-      <c r="R87" s="92"/>
-      <c r="S87" s="92"/>
-      <c r="T87" s="92"/>
-      <c r="U87" s="92"/>
-      <c r="V87" s="92"/>
-      <c r="W87" s="92"/>
-      <c r="X87" s="92"/>
-      <c r="Y87" s="92"/>
-      <c r="Z87" s="92"/>
-      <c r="AA87" s="92"/>
-      <c r="AB87" s="92"/>
-      <c r="AC87" s="92"/>
-      <c r="AD87" s="92"/>
-      <c r="AE87" s="92"/>
-      <c r="AF87" s="92"/>
-      <c r="AG87" s="92"/>
-      <c r="AH87" s="92"/>
-      <c r="AI87" s="92"/>
-      <c r="AJ87" s="92"/>
-      <c r="AK87" s="92"/>
-      <c r="AL87" s="93"/>
+      <c r="C87" s="101"/>
+      <c r="D87" s="102"/>
+      <c r="E87" s="102"/>
+      <c r="F87" s="102"/>
+      <c r="G87" s="102"/>
+      <c r="H87" s="102"/>
+      <c r="I87" s="102"/>
+      <c r="J87" s="102"/>
+      <c r="K87" s="102"/>
+      <c r="L87" s="102"/>
+      <c r="M87" s="102"/>
+      <c r="N87" s="102"/>
+      <c r="O87" s="102"/>
+      <c r="P87" s="102"/>
+      <c r="Q87" s="102"/>
+      <c r="R87" s="102"/>
+      <c r="S87" s="102"/>
+      <c r="T87" s="102"/>
+      <c r="U87" s="102"/>
+      <c r="V87" s="102"/>
+      <c r="W87" s="102"/>
+      <c r="X87" s="102"/>
+      <c r="Y87" s="102"/>
+      <c r="Z87" s="102"/>
+      <c r="AA87" s="102"/>
+      <c r="AB87" s="102"/>
+      <c r="AC87" s="102"/>
+      <c r="AD87" s="102"/>
+      <c r="AE87" s="102"/>
+      <c r="AF87" s="102"/>
+      <c r="AG87" s="102"/>
+      <c r="AH87" s="102"/>
+      <c r="AI87" s="102"/>
+      <c r="AJ87" s="102"/>
+      <c r="AK87" s="102"/>
+      <c r="AL87" s="103"/>
     </row>
     <row r="88" spans="3:38" ht="11.25" customHeight="1">
       <c r="C88" s="13"/>
@@ -4960,46 +4960,46 @@
       <c r="AL102" s="26"/>
     </row>
     <row r="103" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C103" s="94" t="s">
+      <c r="C103" s="104" t="s">
         <v>23</v>
       </c>
-      <c r="D103" s="95"/>
-      <c r="E103" s="95"/>
-      <c r="F103" s="95"/>
-      <c r="G103" s="95"/>
-      <c r="H103" s="95"/>
-      <c r="I103" s="95"/>
-      <c r="J103" s="95"/>
-      <c r="K103" s="95"/>
-      <c r="L103" s="95"/>
-      <c r="M103" s="95"/>
-      <c r="N103" s="95"/>
-      <c r="O103" s="95"/>
-      <c r="P103" s="95"/>
-      <c r="Q103" s="95"/>
-      <c r="R103" s="95"/>
-      <c r="S103" s="95"/>
-      <c r="T103" s="96"/>
-      <c r="U103" s="97" t="s">
+      <c r="D103" s="105"/>
+      <c r="E103" s="105"/>
+      <c r="F103" s="105"/>
+      <c r="G103" s="105"/>
+      <c r="H103" s="105"/>
+      <c r="I103" s="105"/>
+      <c r="J103" s="105"/>
+      <c r="K103" s="105"/>
+      <c r="L103" s="105"/>
+      <c r="M103" s="105"/>
+      <c r="N103" s="105"/>
+      <c r="O103" s="105"/>
+      <c r="P103" s="105"/>
+      <c r="Q103" s="105"/>
+      <c r="R103" s="105"/>
+      <c r="S103" s="105"/>
+      <c r="T103" s="106"/>
+      <c r="U103" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="V103" s="98"/>
-      <c r="W103" s="98"/>
-      <c r="X103" s="98"/>
-      <c r="Y103" s="98"/>
-      <c r="Z103" s="98"/>
-      <c r="AA103" s="98"/>
-      <c r="AB103" s="98"/>
-      <c r="AC103" s="98"/>
-      <c r="AD103" s="98"/>
-      <c r="AE103" s="98"/>
-      <c r="AF103" s="98"/>
-      <c r="AG103" s="98"/>
-      <c r="AH103" s="98"/>
-      <c r="AI103" s="98"/>
-      <c r="AJ103" s="98"/>
-      <c r="AK103" s="98"/>
-      <c r="AL103" s="99"/>
+      <c r="V103" s="108"/>
+      <c r="W103" s="108"/>
+      <c r="X103" s="108"/>
+      <c r="Y103" s="108"/>
+      <c r="Z103" s="108"/>
+      <c r="AA103" s="108"/>
+      <c r="AB103" s="108"/>
+      <c r="AC103" s="108"/>
+      <c r="AD103" s="108"/>
+      <c r="AE103" s="108"/>
+      <c r="AF103" s="108"/>
+      <c r="AG103" s="108"/>
+      <c r="AH103" s="108"/>
+      <c r="AI103" s="108"/>
+      <c r="AJ103" s="108"/>
+      <c r="AK103" s="108"/>
+      <c r="AL103" s="109"/>
     </row>
     <row r="104" spans="3:38" ht="11.25" customHeight="1">
       <c r="C104" s="13"/>
@@ -5364,46 +5364,46 @@
       <c r="AL118" s="26"/>
     </row>
     <row r="119" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C119" s="100" t="s">
+      <c r="C119" s="110" t="s">
         <v>25</v>
       </c>
-      <c r="D119" s="101"/>
-      <c r="E119" s="101"/>
-      <c r="F119" s="101"/>
-      <c r="G119" s="101"/>
-      <c r="H119" s="101"/>
-      <c r="I119" s="101"/>
-      <c r="J119" s="101"/>
-      <c r="K119" s="101"/>
-      <c r="L119" s="101"/>
-      <c r="M119" s="101"/>
-      <c r="N119" s="101"/>
-      <c r="O119" s="101"/>
-      <c r="P119" s="101"/>
-      <c r="Q119" s="101"/>
-      <c r="R119" s="101"/>
-      <c r="S119" s="101"/>
-      <c r="T119" s="102"/>
-      <c r="U119" s="100" t="s">
+      <c r="D119" s="111"/>
+      <c r="E119" s="111"/>
+      <c r="F119" s="111"/>
+      <c r="G119" s="111"/>
+      <c r="H119" s="111"/>
+      <c r="I119" s="111"/>
+      <c r="J119" s="111"/>
+      <c r="K119" s="111"/>
+      <c r="L119" s="111"/>
+      <c r="M119" s="111"/>
+      <c r="N119" s="111"/>
+      <c r="O119" s="111"/>
+      <c r="P119" s="111"/>
+      <c r="Q119" s="111"/>
+      <c r="R119" s="111"/>
+      <c r="S119" s="111"/>
+      <c r="T119" s="112"/>
+      <c r="U119" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="V119" s="101"/>
-      <c r="W119" s="101"/>
-      <c r="X119" s="101"/>
-      <c r="Y119" s="101"/>
-      <c r="Z119" s="101"/>
-      <c r="AA119" s="101"/>
-      <c r="AB119" s="101"/>
-      <c r="AC119" s="101"/>
-      <c r="AD119" s="101"/>
-      <c r="AE119" s="101"/>
-      <c r="AF119" s="101"/>
-      <c r="AG119" s="101"/>
-      <c r="AH119" s="101"/>
-      <c r="AI119" s="101"/>
-      <c r="AJ119" s="101"/>
-      <c r="AK119" s="101"/>
-      <c r="AL119" s="102"/>
+      <c r="V119" s="111"/>
+      <c r="W119" s="111"/>
+      <c r="X119" s="111"/>
+      <c r="Y119" s="111"/>
+      <c r="Z119" s="111"/>
+      <c r="AA119" s="111"/>
+      <c r="AB119" s="111"/>
+      <c r="AC119" s="111"/>
+      <c r="AD119" s="111"/>
+      <c r="AE119" s="111"/>
+      <c r="AF119" s="111"/>
+      <c r="AG119" s="111"/>
+      <c r="AH119" s="111"/>
+      <c r="AI119" s="111"/>
+      <c r="AJ119" s="111"/>
+      <c r="AK119" s="111"/>
+      <c r="AL119" s="112"/>
     </row>
     <row r="120" spans="3:38" ht="11.25" customHeight="1">
       <c r="C120" s="13"/>
@@ -5560,46 +5560,46 @@
       <c r="AL134" s="23"/>
     </row>
     <row r="135" spans="3:38" ht="11.25" customHeight="1">
-      <c r="C135" s="81" t="s">
+      <c r="C135" s="92" t="s">
         <v>18</v>
       </c>
-      <c r="D135" s="82"/>
-      <c r="E135" s="82"/>
-      <c r="F135" s="82"/>
-      <c r="G135" s="82"/>
-      <c r="H135" s="82"/>
-      <c r="I135" s="82"/>
-      <c r="J135" s="82"/>
-      <c r="K135" s="82"/>
-      <c r="L135" s="82"/>
-      <c r="M135" s="82"/>
-      <c r="N135" s="82"/>
-      <c r="O135" s="82"/>
-      <c r="P135" s="82"/>
-      <c r="Q135" s="82"/>
-      <c r="R135" s="82"/>
-      <c r="S135" s="82"/>
-      <c r="T135" s="83"/>
-      <c r="U135" s="84" t="s">
+      <c r="D135" s="93"/>
+      <c r="E135" s="93"/>
+      <c r="F135" s="93"/>
+      <c r="G135" s="93"/>
+      <c r="H135" s="93"/>
+      <c r="I135" s="93"/>
+      <c r="J135" s="93"/>
+      <c r="K135" s="93"/>
+      <c r="L135" s="93"/>
+      <c r="M135" s="93"/>
+      <c r="N135" s="93"/>
+      <c r="O135" s="93"/>
+      <c r="P135" s="93"/>
+      <c r="Q135" s="93"/>
+      <c r="R135" s="93"/>
+      <c r="S135" s="93"/>
+      <c r="T135" s="94"/>
+      <c r="U135" s="95" t="s">
         <v>26</v>
       </c>
-      <c r="V135" s="85"/>
-      <c r="W135" s="85"/>
-      <c r="X135" s="85"/>
-      <c r="Y135" s="85"/>
-      <c r="Z135" s="85"/>
-      <c r="AA135" s="85"/>
-      <c r="AB135" s="85"/>
-      <c r="AC135" s="85"/>
-      <c r="AD135" s="85"/>
-      <c r="AE135" s="85"/>
-      <c r="AF135" s="85"/>
-      <c r="AG135" s="85"/>
-      <c r="AH135" s="85"/>
-      <c r="AI135" s="85"/>
-      <c r="AJ135" s="85"/>
-      <c r="AK135" s="85"/>
-      <c r="AL135" s="86"/>
+      <c r="V135" s="96"/>
+      <c r="W135" s="96"/>
+      <c r="X135" s="96"/>
+      <c r="Y135" s="96"/>
+      <c r="Z135" s="96"/>
+      <c r="AA135" s="96"/>
+      <c r="AB135" s="96"/>
+      <c r="AC135" s="96"/>
+      <c r="AD135" s="96"/>
+      <c r="AE135" s="96"/>
+      <c r="AF135" s="96"/>
+      <c r="AG135" s="96"/>
+      <c r="AH135" s="96"/>
+      <c r="AI135" s="96"/>
+      <c r="AJ135" s="96"/>
+      <c r="AK135" s="96"/>
+      <c r="AL135" s="97"/>
     </row>
     <row r="136" spans="3:38" ht="11.25" customHeight="1"/>
     <row r="137" spans="3:38" ht="11.25" customHeight="1"/>
@@ -5705,21 +5705,59 @@
     <row r="206" ht="11.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="AC2:AM2"/>
-    <mergeCell ref="AC3:AM3"/>
-    <mergeCell ref="AC4:AM4"/>
-    <mergeCell ref="AC5:AM5"/>
-    <mergeCell ref="AC6:AM6"/>
-    <mergeCell ref="U14:AL14"/>
-    <mergeCell ref="O17:S17"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="AI12:AL12"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="C14:T14"/>
-    <mergeCell ref="R12:U12"/>
+    <mergeCell ref="Q45:S45"/>
+    <mergeCell ref="K48:S48"/>
+    <mergeCell ref="K47:S47"/>
+    <mergeCell ref="H46:S46"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="F38:H38"/>
+    <mergeCell ref="P43:S43"/>
+    <mergeCell ref="Q44:S44"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="F43:K43"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="L40:N40"/>
+    <mergeCell ref="O39:Q39"/>
+    <mergeCell ref="L39:N39"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="F39:H39"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="O40:Q40"/>
+    <mergeCell ref="O38:Q38"/>
+    <mergeCell ref="C135:T135"/>
+    <mergeCell ref="U135:AL135"/>
+    <mergeCell ref="AI84:AL84"/>
+    <mergeCell ref="C86:AL87"/>
+    <mergeCell ref="C103:T103"/>
+    <mergeCell ref="U103:AL103"/>
+    <mergeCell ref="C119:T119"/>
+    <mergeCell ref="U119:AL119"/>
+    <mergeCell ref="C84:F84"/>
+    <mergeCell ref="G84:Q84"/>
+    <mergeCell ref="R84:U84"/>
+    <mergeCell ref="V84:AE84"/>
+    <mergeCell ref="AF84:AH84"/>
+    <mergeCell ref="E81:AJ81"/>
+    <mergeCell ref="C83:F83"/>
+    <mergeCell ref="G83:Q83"/>
+    <mergeCell ref="R83:U83"/>
+    <mergeCell ref="V83:AE83"/>
+    <mergeCell ref="AF83:AH83"/>
+    <mergeCell ref="AI83:AL83"/>
     <mergeCell ref="V11:AE11"/>
     <mergeCell ref="V12:AE12"/>
     <mergeCell ref="H19:J19"/>
@@ -5736,59 +5774,21 @@
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="C12:F12"/>
     <mergeCell ref="R11:U11"/>
-    <mergeCell ref="E81:AJ81"/>
-    <mergeCell ref="C83:F83"/>
-    <mergeCell ref="G83:Q83"/>
-    <mergeCell ref="R83:U83"/>
-    <mergeCell ref="V83:AE83"/>
-    <mergeCell ref="AF83:AH83"/>
-    <mergeCell ref="AI83:AL83"/>
-    <mergeCell ref="C135:T135"/>
-    <mergeCell ref="U135:AL135"/>
-    <mergeCell ref="AI84:AL84"/>
-    <mergeCell ref="C86:AL87"/>
-    <mergeCell ref="C103:T103"/>
-    <mergeCell ref="U103:AL103"/>
-    <mergeCell ref="C119:T119"/>
-    <mergeCell ref="U119:AL119"/>
-    <mergeCell ref="C84:F84"/>
-    <mergeCell ref="G84:Q84"/>
-    <mergeCell ref="R84:U84"/>
-    <mergeCell ref="V84:AE84"/>
-    <mergeCell ref="AF84:AH84"/>
-    <mergeCell ref="F39:H39"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="O40:Q40"/>
-    <mergeCell ref="O38:Q38"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="L40:N40"/>
-    <mergeCell ref="O39:Q39"/>
-    <mergeCell ref="L39:N39"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="F38:H38"/>
-    <mergeCell ref="P43:S43"/>
-    <mergeCell ref="Q44:S44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="F43:K43"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="L38:N38"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="Q45:S45"/>
-    <mergeCell ref="K48:S48"/>
-    <mergeCell ref="K47:S47"/>
-    <mergeCell ref="H46:S46"/>
-    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="U14:AL14"/>
+    <mergeCell ref="O17:S17"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="AI12:AL12"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="C14:T14"/>
+    <mergeCell ref="R12:U12"/>
+    <mergeCell ref="AC2:AM2"/>
+    <mergeCell ref="AC3:AM3"/>
+    <mergeCell ref="AC4:AM4"/>
+    <mergeCell ref="AC5:AM5"/>
+    <mergeCell ref="AC6:AM6"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>